<commit_message>
homologizer ruzne kombinace na zkousku
</commit_message>
<xml_diff>
--- a/homologizer/scripts/data/target_samples-upravenypodlevysledkuss.csv.xlsx
+++ b/homologizer/scripts/data/target_samples-upravenypodlevysledkuss.csv.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rycht\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rycht\Documents\homologizer_aconitum\homologizer\scripts\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1D51D39A-E307-4AEB-A493-D22C9F312512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6012E62-201F-4A51-8143-1EC698896EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29550" yWindow="-5210" windowWidth="12240" windowHeight="14170" xr2:uid="{05706F9B-7D61-4D2F-8007-4F44AD4A6C21}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{05706F9B-7D61-4D2F-8007-4F44AD4A6C21}"/>
   </bookViews>
   <sheets>
     <sheet name="target_samples" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>vzorek</t>
   </si>
@@ -167,13 +167,175 @@
   </si>
   <si>
     <t>n_FRS8_088</t>
+  </si>
+  <si>
+    <t>b_TNB8_064</t>
+  </si>
+  <si>
+    <t>c_MDKH2_074</t>
+  </si>
+  <si>
+    <t>c_MDKH8_075</t>
+  </si>
+  <si>
+    <t>c_PJS1_180</t>
+  </si>
+  <si>
+    <t>c_PJS2_181</t>
+  </si>
+  <si>
+    <t>c_RHSK1_182</t>
+  </si>
+  <si>
+    <t>deg_UMA1_111</t>
+  </si>
+  <si>
+    <t>e_OLS17_013</t>
+  </si>
+  <si>
+    <t>e_OLS3_126</t>
+  </si>
+  <si>
+    <t>las_PLSK1_168</t>
+  </si>
+  <si>
+    <t>lyc_OLS1_183</t>
+  </si>
+  <si>
+    <t>n_BNFA8_033</t>
+  </si>
+  <si>
+    <t>n_CHA1_073</t>
+  </si>
+  <si>
+    <t>n_CHA2_107</t>
+  </si>
+  <si>
+    <t>n_CHA3_108</t>
+  </si>
+  <si>
+    <t>n_CHA4_110</t>
+  </si>
+  <si>
+    <t>n_DEU8_026</t>
+  </si>
+  <si>
+    <t>n_DPK10_038</t>
+  </si>
+  <si>
+    <t>n_HPSK1_174</t>
+  </si>
+  <si>
+    <t>n_HPSK2_175</t>
+  </si>
+  <si>
+    <t>n_JIZ2_018</t>
+  </si>
+  <si>
+    <t>n_JIZ5_160</t>
+  </si>
+  <si>
+    <t>n_JIZ7_019</t>
+  </si>
+  <si>
+    <t>n_KKS2_103</t>
+  </si>
+  <si>
+    <t>n_KKS5_167</t>
+  </si>
+  <si>
+    <t>n_KKS8_104</t>
+  </si>
+  <si>
+    <t>n_KPJ1_043</t>
+  </si>
+  <si>
+    <t>n_KPS2_091</t>
+  </si>
+  <si>
+    <t>n_KPS5_158</t>
+  </si>
+  <si>
+    <t>n_KPS8_092</t>
+  </si>
+  <si>
+    <t>n_KVIS2_001</t>
+  </si>
+  <si>
+    <t>n_KVIS8_002</t>
+  </si>
+  <si>
+    <t>n_KVS5_155</t>
+  </si>
+  <si>
+    <t>n_LBK10_042</t>
+  </si>
+  <si>
+    <t>n_LBK1_041</t>
+  </si>
+  <si>
+    <t>n_LBK5_159</t>
+  </si>
+  <si>
+    <t>n_LNSA2_034</t>
+  </si>
+  <si>
+    <t>n_LNSA5_132</t>
+  </si>
+  <si>
+    <t>n_LNSA8_035</t>
+  </si>
+  <si>
+    <t>n_LSA5_130</t>
+  </si>
+  <si>
+    <t>n_LSRA2_027</t>
+  </si>
+  <si>
+    <t>n_LSRA8_028</t>
+  </si>
+  <si>
+    <t>n_LZS1_116</t>
+  </si>
+  <si>
+    <t>n_LZS4_152</t>
+  </si>
+  <si>
+    <t>n_LZS8_117</t>
+  </si>
+  <si>
+    <t>n_MDS2_003</t>
+  </si>
+  <si>
+    <t>n_MDS5_156</t>
+  </si>
+  <si>
+    <t>n_MDS8_004</t>
+  </si>
+  <si>
+    <t>n_MFSK1_022</t>
+  </si>
+  <si>
+    <t>n_MJS1_149</t>
+  </si>
+  <si>
+    <t>n_MJS2_081</t>
+  </si>
+  <si>
+    <t>n_MKJ10_046</t>
+  </si>
+  <si>
+    <t>n_MKJ1_044</t>
+  </si>
+  <si>
+    <t>n_MKJ5_045</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,6 +486,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -668,8 +836,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % – Zvýraznění 1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1045,10 +1216,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3049AB4-D770-4807-986B-03DD6C7E1CE6}">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1070,220 +1242,220 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
+        <v>49</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1">
+        <v>3</v>
       </c>
       <c r="D2">
         <v>3</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
+        <v>50</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
+        <v>51</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
+        <v>52</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
+        <v>53</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1">
         <v>3</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7">
+        <v>54</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
+        <v>55</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14">
         <v>4</v>
@@ -1291,16 +1463,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15">
         <v>4</v>
@@ -1308,16 +1480,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E16">
         <v>4</v>
@@ -1325,16 +1497,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17">
         <v>4</v>
@@ -1342,16 +1514,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18">
         <v>4</v>
@@ -1359,16 +1531,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19">
         <v>4</v>
@@ -1376,7 +1548,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -1385,7 +1557,7 @@
         <v>2</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E20">
         <v>4</v>
@@ -1393,7 +1565,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1410,16 +1582,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22">
         <v>4</v>
@@ -1427,16 +1599,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -1444,7 +1616,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -1453,7 +1625,7 @@
         <v>2</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E24">
         <v>4</v>
@@ -1461,13 +1633,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -1478,16 +1650,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26">
         <v>4</v>
@@ -1495,16 +1667,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27">
         <v>4</v>
@@ -1512,7 +1684,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B28">
         <v>1</v>
@@ -1529,16 +1701,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E29">
         <v>4</v>
@@ -1546,7 +1718,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -1555,7 +1727,7 @@
         <v>3</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30">
         <v>4</v>
@@ -1563,10 +1735,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31">
         <v>3</v>
@@ -1580,10 +1752,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -1597,7 +1769,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B33">
         <v>1</v>
@@ -1606,7 +1778,7 @@
         <v>2</v>
       </c>
       <c r="D33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E33">
         <v>4</v>
@@ -1614,10 +1786,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -1631,16 +1803,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E35">
         <v>4</v>
@@ -1648,7 +1820,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -1665,16 +1837,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37">
         <v>2</v>
       </c>
       <c r="D37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -1682,16 +1854,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38">
         <v>4</v>
@@ -1699,13 +1871,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B39">
         <v>2</v>
       </c>
       <c r="C39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -1716,13 +1888,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D40">
         <v>3</v>
@@ -1733,7 +1905,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -1750,16 +1922,16 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D42">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E42">
         <v>4</v>
@@ -1767,16 +1939,16 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43">
         <v>4</v>
@@ -1784,16 +1956,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44">
         <v>4</v>
@@ -1801,18 +1973,936 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45">
+        <v>3</v>
+      </c>
+      <c r="E45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="D46">
+        <v>3</v>
+      </c>
+      <c r="E46">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+      <c r="D47">
+        <v>3</v>
+      </c>
+      <c r="E47">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+      <c r="D49">
+        <v>3</v>
+      </c>
+      <c r="E49">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50">
+        <v>3</v>
+      </c>
+      <c r="E50">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>39</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>2</v>
+      </c>
+      <c r="E51">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>40</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+      <c r="E52">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>41</v>
+      </c>
+      <c r="B53">
+        <v>2</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53">
+        <v>3</v>
+      </c>
+      <c r="E53">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54">
+        <v>2</v>
+      </c>
+      <c r="D54">
+        <v>3</v>
+      </c>
+      <c r="E54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55">
+        <v>2</v>
+      </c>
+      <c r="D55">
+        <v>2</v>
+      </c>
+      <c r="E55">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56">
+        <v>2</v>
+      </c>
+      <c r="D56">
+        <v>3</v>
+      </c>
+      <c r="E56">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>43</v>
+      </c>
+      <c r="B57">
+        <v>2</v>
+      </c>
+      <c r="C57">
+        <v>3</v>
+      </c>
+      <c r="D57">
+        <v>4</v>
+      </c>
+      <c r="E57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>44</v>
+      </c>
+      <c r="B58">
+        <v>2</v>
+      </c>
+      <c r="C58">
+        <v>3</v>
+      </c>
+      <c r="D58">
+        <v>3</v>
+      </c>
+      <c r="E58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>45</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59">
+        <v>2</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
+      </c>
+      <c r="E59">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>46</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60">
+        <v>3</v>
+      </c>
+      <c r="D60">
+        <v>4</v>
+      </c>
+      <c r="E60">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>47</v>
+      </c>
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61">
+        <v>3</v>
+      </c>
+      <c r="D61">
+        <v>3</v>
+      </c>
+      <c r="E61">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62">
+        <v>2</v>
+      </c>
+      <c r="D62">
+        <v>4</v>
+      </c>
+      <c r="E62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+      <c r="D63">
+        <v>4</v>
+      </c>
+      <c r="E63">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="D64">
+        <v>4</v>
+      </c>
+      <c r="E64">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65">
+        <v>3</v>
+      </c>
+      <c r="D65">
+        <v>3</v>
+      </c>
+      <c r="E65">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66">
+        <v>2</v>
+      </c>
+      <c r="D66">
+        <v>4</v>
+      </c>
+      <c r="E66">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="D67">
+        <v>3</v>
+      </c>
+      <c r="E67">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>72</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68">
+        <v>2</v>
+      </c>
+      <c r="D68">
+        <v>4</v>
+      </c>
+      <c r="E68">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>73</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69">
+        <v>4</v>
+      </c>
+      <c r="E69">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70">
+        <v>2</v>
+      </c>
+      <c r="D70">
+        <v>4</v>
+      </c>
+      <c r="E70">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>75</v>
+      </c>
+      <c r="B71">
+        <v>2</v>
+      </c>
+      <c r="C71">
+        <v>2</v>
+      </c>
+      <c r="D71">
+        <v>4</v>
+      </c>
+      <c r="E71">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>76</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72">
+        <v>2</v>
+      </c>
+      <c r="D72">
+        <v>3</v>
+      </c>
+      <c r="E72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>77</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73">
+        <v>2</v>
+      </c>
+      <c r="D73">
+        <v>4</v>
+      </c>
+      <c r="E73">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>78</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74">
+        <v>2</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+      <c r="E74">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>79</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75">
+        <v>2</v>
+      </c>
+      <c r="D75">
+        <v>2</v>
+      </c>
+      <c r="E75">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76">
+        <v>3</v>
+      </c>
+      <c r="D76">
+        <v>3</v>
+      </c>
+      <c r="E76">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>81</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="C77">
+        <v>3</v>
+      </c>
+      <c r="D77">
+        <v>4</v>
+      </c>
+      <c r="E77">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>82</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+      <c r="C78">
+        <v>2</v>
+      </c>
+      <c r="D78">
+        <v>4</v>
+      </c>
+      <c r="E78">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>83</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79">
+        <v>3</v>
+      </c>
+      <c r="D79">
+        <v>3</v>
+      </c>
+      <c r="E79">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>84</v>
+      </c>
+      <c r="B80">
+        <v>2</v>
+      </c>
+      <c r="C80">
+        <v>3</v>
+      </c>
+      <c r="D80">
+        <v>3</v>
+      </c>
+      <c r="E80">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+      <c r="B81">
+        <v>2</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81">
+        <v>2</v>
+      </c>
+      <c r="E81">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>86</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82">
+        <v>4</v>
+      </c>
+      <c r="E82">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>87</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83">
+        <v>3</v>
+      </c>
+      <c r="D83">
+        <v>3</v>
+      </c>
+      <c r="E83">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>88</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84">
+        <v>2</v>
+      </c>
+      <c r="D84">
+        <v>4</v>
+      </c>
+      <c r="E84">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>89</v>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+      <c r="C85">
+        <v>3</v>
+      </c>
+      <c r="D85">
+        <v>4</v>
+      </c>
+      <c r="E85">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>90</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86">
+        <v>2</v>
+      </c>
+      <c r="D86">
+        <v>2</v>
+      </c>
+      <c r="E86">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>91</v>
+      </c>
+      <c r="B87">
+        <v>2</v>
+      </c>
+      <c r="C87">
+        <v>3</v>
+      </c>
+      <c r="D87">
+        <v>3</v>
+      </c>
+      <c r="E87">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>92</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88">
+        <v>2</v>
+      </c>
+      <c r="D88">
+        <v>2</v>
+      </c>
+      <c r="E88">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>93</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89">
+        <v>2</v>
+      </c>
+      <c r="D89">
+        <v>3</v>
+      </c>
+      <c r="E89">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>94</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90">
+        <v>2</v>
+      </c>
+      <c r="D90">
+        <v>2</v>
+      </c>
+      <c r="E90">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91">
+        <v>2</v>
+      </c>
+      <c r="C91">
+        <v>2</v>
+      </c>
+      <c r="D91">
+        <v>2</v>
+      </c>
+      <c r="E91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>96</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92">
+        <v>2</v>
+      </c>
+      <c r="D92">
+        <v>2</v>
+      </c>
+      <c r="E92">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>97</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93">
+        <v>3</v>
+      </c>
+      <c r="D93">
+        <v>3</v>
+      </c>
+      <c r="E93">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>98</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
+      </c>
+      <c r="D94">
+        <v>3</v>
+      </c>
+      <c r="E94">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>99</v>
+      </c>
+      <c r="B95">
+        <v>1</v>
+      </c>
+      <c r="C95">
+        <v>2</v>
+      </c>
+      <c r="D95">
+        <v>4</v>
+      </c>
+      <c r="E95">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>100</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+      <c r="C96">
+        <v>2</v>
+      </c>
+      <c r="D96">
+        <v>2</v>
+      </c>
+      <c r="E96">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>101</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97">
+        <v>2</v>
+      </c>
+      <c r="D97">
+        <v>4</v>
+      </c>
+      <c r="E97">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>102</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98">
+        <v>2</v>
+      </c>
+      <c r="D98">
+        <v>2</v>
+      </c>
+      <c r="E98">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
         <v>5</v>
       </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-      <c r="D45">
-        <v>3</v>
-      </c>
-      <c r="E45">
+      <c r="B99">
+        <v>1</v>
+      </c>
+      <c r="C99">
+        <v>1</v>
+      </c>
+      <c r="D99">
+        <v>3</v>
+      </c>
+      <c r="E99">
         <v>4</v>
       </c>
     </row>

</xml_diff>